<commit_message>
feat(F-NAR-019): ATOM-COL.POL.001-10 Le croissant d'Amir
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.POL.001-10.xlsx
+++ b/stories/arbres/ATOM-COL.POL.001-10.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le croissant du bout d'Amir</t>
+          <t>Le croissant d'Amir</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>paillasson mouillé, boulangerie le matin</t>
+          <t>boulangerie, corbeille d'osier, vitrine, sésame, marbre, cloche</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut le croissant du bout de la rangée. Il dit bonjour, s'il te plaît, merci. Une miette dorée reste sur sa manche.</t>
+          <t>Une graine de sésame tape le marbre. Sur l'osier, un éclat de corbeille brille. Amir veut le croissant au sésame maintenant. Il parle trop vite, sans le mot : la dame ne lève pas les yeux. Il refuse de foncer, dit bonjour, s'il te plaît, obtient le sachet. Merci vécu. Un sachet trop vite : les graines tombent. Un éclat de corbeille reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le paillasson sent encore la pluie. Les lacets d'Amir laissent deux traits mouillés. Derrière la porte, le four souffle. Ça sent le beurre, déjà. Papa porte un journal encore un peu humide. Le papier du journal sent l'encre. Tes lacets sont mouillés, Amir. Ils tapent, maman. Deux petits tap-tap. On les entend, hein ? Oui. De la vapeur colle à la vitre, en bas. Un croissant s'y dessine, un peu flou. Celui du bout. On montre celui du bout. En ce moment, Amir pose le pied. Le paillasson est rêche, un peu chaud. Maman pousse la porte. Une cloche fait ding. L'air sent le beurre et le pain. Les croissants sont dorés, en rang. Ils sont tous pareils. Sauf celui du bout. Il est plus brun. La dame essuie une miette sur le marbre. Elle a le torchon. On la laisse finir. La miette part. La dame lève les yeux. Amir montre le croissant du bout. Tu demandes, Amir.</t>
+          <t>Une graine de sésame tape le marbre. Elle roule près de l'osier. Amir connaît cette odeur de beurre. La corbeille d'osier paraît neuve. Sur l'osier, un éclat de corbeille brille. Il brille, papa. Tu le vois, sur l'osier ? Amir touche l'éclat de corbeille, un instant. L'osier pique un peu le doigt. Il est rêche. Le col, un bouton de plus. Voilà. Le soleil pose un carré sur le marbre. Il est jaune. On avance. La vitrine tient des pains dorés. Des graines collent à la vitrine. Ça sent le beurre ! Tu sens, Amir ? Oui. Une odeur de sésame arrive. Ça sent les graines. Tu restes près de nous ? Oui, maman. La porte de bois attend. On entre. Une petite cloche fait ding. L'air chaud touche les joues. J'ai les joues chaudes. En ce moment, Amir serre le manteau. Le marbre est froid sous ses doigts. La dame range la corbeille d'osier. Des croissants dorés dorment dans l'osier. Je le veux, maintenant. On s'approche du bois. Celui du bout ! Un croissant au sésame attend au bout. Amir parle trop vite vers l'osier. Les mots se perdent dans la cloche. Oh. La dame ne lève pas les yeux. Ses mains tiennent la corbeille. Je le prends ! Le croissant reste dans l'osier. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Les épaules d'Amir tombent un peu. Ça serre, dans son ventre. Le croissant est dans l'osier. Tu le vois, Amir ? Papa se baisse à sa hauteur. Tu parles à la dame, Amir. Elle t'écoute, Amir ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le paillasson sent encore la pluie. Les lacets d'Amir laissent deux traits mouillés. Derrière la porte, le four souffle. Ça sent le beurre, déjà. Papa porte un journal encore un peu humide. Le papier du journal sent l'encre. Tes lacets sont mouillés, Amir. Ils tapent, maman. Deux petits tap-tap. On les entend, hein ? Oui. De la vapeur colle à la vitre, en bas. Un croissant s'y dessine, un peu flou. Celui du bout. On montre celui du bout. En ce moment, Amir pose le pied. Le paillasson est rêche, un peu chaud. Maman pousse la porte. Une cloche fait ding. L'air sent le beurre et le pain. Les croissants sont dorés, en rang. Ils sont tous pareils. Sauf celui du bout. Il est plus brun. La dame essuie une miette sur le marbre. Elle a le torchon. On la laisse finir. La miette part. La dame lève les yeux. Amir montre le croissant du bout. Tu demandes, Amir.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une graine de sésame tape le marbre. Elle roule près de l'osier. Amir connaît cette odeur de beurre. La corbeille d'osier paraît neuve. Sur l'osier, un &lt;emphasis level="moderate"&gt;éclat de corbeille&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, sur l'osier ? Amir touche l'éclat de corbeille, un instant. L'osier pique un peu le doigt. Il est rêche. Le col, un bouton de plus. Voilà. Le soleil pose un carré sur le marbre. Il est jaune. On avance. La vitrine tient des pains dorés. Des graines collent à la vitrine. Ça sent le beurre ! Tu sens, Amir ? Oui. Une odeur de sésame arrive. Ça sent les graines. Tu restes près de nous ? Oui, maman. La porte de bois attend. On entre. Une petite cloche fait ding. L'air chaud touche les joues. J'ai les joues chaudes. En ce moment, Amir serre le manteau. Le marbre est froid sous ses doigts. La dame range la corbeille d'osier. Des croissants dorés dorment dans l'osier. Je le veux, maintenant. On s'approche du bois. Celui du bout ! Un croissant au sésame attend au bout. Amir parle trop vite vers l'osier. Les mots se perdent dans la cloche. Oh. La dame ne lève pas les yeux. Ses mains tiennent la corbeille. Je le prends ! Le croissant reste dans l'osier. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Les épaules d'Amir tombent un peu. Ça serre, dans son ventre. Le croissant est dans l'osier. Tu le vois, Amir ? Papa se baisse à sa hauteur. Tu parles à la dame, Amir. Elle t'écoute, Amir ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Félix entre à la boulangerie. Maman est avec lui. Il sent le pain chaud. Félix dit : &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. La dame sourit. Maman dit : on demande. Félix dit : un croissant, s'il te plaît. La dame tend le sac. Le sac est chaud. Félix dit : merci. Maman dit : bonjour, s'il te plaît, merci. Félix répète. Bonjour. S'il te plaît. Merci. Ils sortent. Félix tient le sac. Le croissant sent le beurre. Maman sourit. Félix a dit les trois mots.&lt;/slow&gt; [pause]</t>
+          <t>Une graine de sésame tape le marbre. Elle roule près de l'osier. Amir connaît cette odeur de beurre. La corbeille d'osier paraît neuve. Sur l'osier, un &lt;emphasis&gt;éclat de corbeille&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, sur l'osier ? Amir touche l'éclat de corbeille, un instant. L'osier pique un peu le doigt. Il est rêche. Le col, un bouton de plus. Voilà. Le soleil pose un carré sur le marbre. Il est jaune. On avance. La vitrine tient des pains dorés. Des graines collent à la vitrine. Ça sent le beurre ! Tu sens, Amir ? Oui. Une odeur de sésame arrive. Ça sent les graines. Tu restes près de nous ? Oui, maman. La porte de bois attend. On entre. Une petite cloche fait ding. L'air chaud touche les joues. J'ai les joues chaudes. En ce moment, Amir serre le manteau. Le marbre est froid sous ses doigts. La dame range la corbeille d'osier. Des croissants dorés dorment dans l'osier. Je le veux, maintenant. On s'approche du bois. Celui du bout ! Un croissant au sésame attend au bout. Amir parle trop vite vers l'osier. Les mots se perdent dans la cloche. Oh. La dame ne lève pas les yeux. Ses mains tiennent la corbeille. Je le prends ! Le croissant reste dans l'osier. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Les épaules d'Amir tombent un peu. Ça serre, dans son ventre. Le croissant est dans l'osier. Tu le vois, Amir ? Papa se baisse à sa hauteur. Tu parles à la dame, Amir. Elle t'écoute, Amir ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>éclat de corbeille</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,47 +1324,73 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_croissant_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le paillasson sent encore la pluie.
-narrateur|Les lacets d'Amir laissent deux traits mouillés.
-narrateur|Derrière la porte, le four souffle.
-narrateur|Ça sent le beurre, déjà.
-narrateur|Papa porte un journal encore un peu humide.
-narrateur|Le papier du journal sent l'encre.
-maman|Tes lacets sont mouillés, Amir.
-enfant-m|Ils tapent, maman.
-papa|Deux petits tap-tap.
-maman|On les entend, hein ?
+          <t>narrateur|Une graine de sésame tape le marbre.
+narrateur|Elle roule près de l'osier.
+narrateur|Amir connaît cette odeur de beurre.
+narrateur|La corbeille d'osier paraît neuve.
+narrateur|Sur l'osier, un éclat de corbeille brille.
+enfant-m|Il brille, papa.
+papa|Tu le vois, sur l'osier ?
+narrateur|Amir touche l'éclat de corbeille, un instant.
+narrateur|L'osier pique un peu le doigt.
+enfant-m|Il est rêche.
+maman|Le col, un bouton de plus.
+papa|Voilà.
+narrateur|Le soleil pose un carré sur le marbre.
+enfant-m|Il est jaune.
+papa|On avance.
+narrateur|La vitrine tient des pains dorés.
+narrateur|Des graines collent à la vitrine.
+enfant-m|Ça sent le beurre !
+maman|Tu sens, Amir ?
 enfant-m|Oui.
-narrateur|De la vapeur colle à la vitre, en bas.
-narrateur|Un croissant s'y dessine, un peu flou.
-enfant-m|Celui du bout.
-papa|On montre celui du bout.
-narrateur|En ce moment, Amir pose le pied.
-narrateur|Le paillasson est rêche, un peu chaud.
-narrateur|Maman pousse la porte.
-narrateur|Une cloche fait ding.
-narrateur|L'air sent le beurre et le pain.
-narrateur|Les croissants sont dorés, en rang.
-enfant-m|Ils sont tous pareils.
-papa|Sauf celui du bout.
-enfant-m|Il est plus brun.
-narrateur|La dame essuie une miette sur le marbre.
-maman|Elle a le torchon.
-papa|On la laisse finir.
-narrateur|La miette part.
-narrateur|La dame lève les yeux.
-narrateur|Amir montre le croissant du bout.
-maman|Tu demandes, Amir.</t>
+narrateur|Une odeur de sésame arrive.
+enfant-m|Ça sent les graines.
+maman|Tu restes près de nous ?
+enfant-m|Oui, maman.
+narrateur|La porte de bois attend.
+papa|On entre.
+narrateur|Une petite cloche fait ding.
+narrateur|L'air chaud touche les joues.
+enfant-m|J'ai les joues chaudes.
+narrateur|En ce moment, Amir serre le manteau.
+narrateur|Le marbre est froid sous ses doigts.
+narrateur|La dame range la corbeille d'osier.
+narrateur|Des croissants dorés dorment dans l'osier.
+enfant-m|Je le veux, maintenant.
+papa|On s'approche du bois.
+enfant-m|Celui du bout !
+narrateur|Un croissant au sésame attend au bout.
+narrateur|Amir parle trop vite vers l'osier.
+narrateur|Les mots se perdent dans la cloche.
+enfant-m|Oh.
+narrateur|La dame ne lève pas les yeux.
+narrateur|Ses mains tiennent la corbeille.
+enfant-m|Je le prends !
+narrateur|Le croissant reste dans l'osier.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Les épaules d'Amir tombent un peu.
+narrateur|Ça serre, dans son ventre.
+maman|Le croissant est dans l'osier.
+papa|Tu le vois, Amir ?
+narrateur|Papa se baisse à sa hauteur.
+maman|Tu parles à la dame, Amir.
+papa|Elle t'écoute, Amir ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>paillasson,cloche</t>
+          <t>cloche,osier</t>
         </is>
       </c>
     </row>
@@ -1391,17 +1417,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Amir veut le croissant. Que dit-il ?</t>
+          <t>Amir parle à la dame. Quels mots dit-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Amir veut le croissant. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Amir parle à la &lt;emphasis level="moderate"&gt;dame&lt;/emphasis&gt;. Quels mots dit-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Félix parle à la dame. Quels mots dit-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Amir parle à la &lt;emphasis&gt;dame&lt;/emphasis&gt;. Quels mots dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1426,7 +1452,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il dit bonjour. Que dit Amir ?</t>
+          <t>Il dit bonjour. Quels mots dit Amir ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1464,7 +1490,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1472,10 +1498,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1490,34 +1516,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>dame</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1526,13 +1556,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1542,13 +1572,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_dit_bonjour_a_la_dame; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Amir veut le croissant.
-narrateur|Que dit-il ?</t>
+          <t>narrateur|Amir parle à la dame.
+narrateur|Quels mots dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1575,17 +1605,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Un croissant, s'il te plaît. Celui du bout. La dame glisse le croissant dans un sac. Le sac est chaud. Le papier craque. Merci. Merci. Amir tient le sac à deux mains. Ça sent le beurre, tout près du nez. Il est chaud, maman. Oui. Une miette sur ta manche. Elle est dorée. Tu la goûtes ? Elle est bonne. Ils restent un moment près de la vitre. Dehors, les lacets ne tapent plus. On rentre ? Oui, papa. Le sac fume un peu, tout doux. Tu le tiens haut ? Oui. Comme ça, il reste chaud.</t>
+          <t>Amir avance trop vite vers l'osier. Celui du bout, maintenant ! Sa voix se mélange à la cloche. Oh. Le croissant reste dans l'osier. Il refuse de foncer. Amir referme la bouche. Il écoute la cloche, un instant. Tu veux venir près de l'osier ? Papa s'accroupit à la même hauteur. Amir pose un pied sur le pas. Le bois est tiède, un peu lisse. Bonjour. Bonjour. Celui du bout, s'il te plaît. La dame tend le croissant. Le papier enveloppe le croissant. Le sachet est chaud contre le manteau. Merci. Merci, Amir. Papa a entendu toute la phrase. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Ça sent le beurre et le sésame. Le croissant est à moi. Il est dans tes mains. Amir pose une main sur le sachet. Le papier est un peu rêche. La cloche se tait. Il est chaud, papa. Tu le portes jusqu'à la rue ? Oui, papa. Des graines tiennent sur le papier.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Un croissant, s'il te plaît. Celui du bout. La dame glisse le croissant dans un sac. Le sac est chaud. Le papier craque. Merci. Merci. Amir tient le sac à deux mains. Ça sent le beurre, tout près du nez. Il est chaud, maman. Oui. Une miette sur ta manche. Elle est dorée. Tu la goûtes ? Elle est bonne. Ils restent un moment près de la vitre. Dehors, les lacets ne tapent plus. On rentre ? Oui, papa. Le sac fume un peu, tout doux. Tu le tiens haut ? Oui. Comme ça, il reste chaud.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir avance trop vite vers l'osier. Celui du bout, maintenant ! Sa voix se mélange à la cloche. Oh. Le croissant reste dans l'osier. Il refuse de foncer. Amir referme la bouche. Il écoute la cloche, un instant. Tu veux venir près de l'osier ? Papa s'accroupit à la même hauteur. Amir pose un pied sur le pas. Le bois est tiède, un peu lisse. &lt;emphasis level="moderate"&gt;Bonjour&lt;/emphasis&gt;. Bonjour. Celui du bout, s'il te plaît. La dame tend le croissant. Le papier enveloppe le croissant. Le sachet est chaud contre le manteau. Merci. Merci, Amir. Papa a entendu toute la phrase. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Ça sent le beurre et le sésame. Le croissant est à moi. Il est dans tes mains. Amir pose une main sur le sachet. Le papier est un peu rêche. La cloche se tait. Il est chaud, papa. Tu le portes jusqu'à la rue ? Oui, papa. Des graines tiennent sur le papier.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Félix a dit &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Il a dit s'il te plaît. Il a dit merci. Maman était là.&lt;/slow&gt; [pause]</t>
+          <t>Amir avance trop vite vers l'osier. Celui du bout, maintenant ! Sa voix se mélange à la cloche. Oh. Le croissant reste dans l'osier. Il refuse de foncer. Amir referme la bouche. Il écoute la cloche, un instant. Tu veux venir près de l'osier ? Papa s'accroupit à la même hauteur. Amir pose un pied sur le pas. Le bois est tiède, un peu lisse. &lt;emphasis&gt;Bonjour&lt;/emphasis&gt;. Bonjour. Celui du bout, s'il te plaît. La dame tend le croissant. Le papier enveloppe le croissant. Le sachet est chaud contre le manteau. Merci. Merci, Amir. Papa a entendu toute la phrase. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Ça sent le beurre et le sésame. Le croissant est à moi. Il est dans tes mains. Amir pose une main sur le sachet. Le papier est un peu rêche. La cloche se tait. Il est chaud, papa. Tu le portes jusqu'à la rue ? Oui, papa. Des graines tiennent sur le papier. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1632,18 +1662,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1666,30 +1696,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>Bonjour</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1698,10 +1728,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1710,45 +1740,55 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=bonjour_s_il_te_plait_merci_vecus; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-m|Bonjour.
+          <t>narrateur|Amir avance trop vite vers l'osier.
+enfant-m|Celui du bout, maintenant !
+narrateur|Sa voix se mélange à la cloche.
+enfant-m|Oh.
+narrateur|Le croissant reste dans l'osier.
+narrateur|Il refuse de foncer.
+narrateur|Amir referme la bouche.
+narrateur|Il écoute la cloche, un instant.
+papa|Tu veux venir près de l'osier ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Amir pose un pied sur le pas.
+narrateur|Le bois est tiède, un peu lisse.
+enfant-m|Bonjour.
 papa|Bonjour.
-enfant-m|Un croissant, s'il te plaît.
-enfant-m|Celui du bout.
-narrateur|La dame glisse le croissant dans un sac.
-narrateur|Le sac est chaud.
-narrateur|Le papier craque.
+enfant-m|Celui du bout, s'il te plaît.
+narrateur|La dame tend le croissant.
+narrateur|Le papier enveloppe le croissant.
+narrateur|Le sachet est chaud contre le manteau.
 enfant-m|Merci.
-maman|Merci.
-narrateur|Amir tient le sac à deux mains.
-narrateur|Ça sent le beurre, tout près du nez.
-enfant-m|Il est chaud, maman.
-maman|Oui.
-papa|Une miette sur ta manche.
-enfant-m|Elle est dorée.
-maman|Tu la goûtes ?
-enfant-m|Elle est bonne.
-narrateur|Ils restent un moment près de la vitre.
-narrateur|Dehors, les lacets ne tapent plus.
-papa|On rentre ?
+papa|Merci, Amir.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre d'Amir se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|Tu as les mains au chaud ?
+enfant-m|Un peu, maman.
+narrateur|Ça sent le beurre et le sésame.
+enfant-m|Le croissant est à moi.
+maman|Il est dans tes mains.
+narrateur|Amir pose une main sur le sachet.
+narrateur|Le papier est un peu rêche.
+narrateur|La cloche se tait.
+enfant-m|Il est chaud, papa.
+papa|Tu le portes jusqu'à la rue ?
 enfant-m|Oui, papa.
-narrateur|Le sac fume un peu, tout doux.
-maman|Tu le tiens haut ?
-enfant-m|Oui.
-papa|Comme ça, il reste chaud.</t>
+narrateur|Des graines tiennent sur le papier.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>papier</t>
+          <t>papier,cloche</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1815,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent le long de la rue mouillée. Le croissant fume encore, tout doux. À la maison, papa ouvre le sac. Le croissant est doré, un peu cassant. Tu veux un bout ? Oui, maman. S'il te plaît. Amir croque. C'est tiède. Ça sent le beurre. Merci, maman. Merci, Amir. Des miettes dorées restent au fond du sac. Tes lacets sèchent, maintenant. Ils ne tapent plus. Non. C'était celui du bout. Oui. Le paillasson, loin, garde encore la pluie. Le journal sèche, lui aussi. Il était mouillé. Un peu, oui.</t>
+          <t>Amir tire le sachet trop vite. Je le mange, d'un coup ! Le papier glisse entre les doigts. Des graines de sésame tombent au marbre. Le croissant penche vers le sol. Oh. Amir avance les mains. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Amir refuse de foncer. Personne ne dit la suite. Amir observe l'osier, écoute la boutique. Sur l'osier, un éclat de corbeille brille. Là, près de la corbeille. Amir tient le sachet des deux mains. Le papier est rêche, un peu chaud. Il est chaud, papa. Tu le portes jusqu'à la porte ? Oui, papa. On sort ? Oui, maman. La porte s'ouvre. La cloche fait ding. L'air plus frais revient sur les joues. Amir serre le sachet contre lui. Il reste chaud. On marche. Le sachet penche, puis se cale. Je le tiens. On avance. Amir passe le pas de bois. Le bois craque, un peu. Les graines sont à moi. Elles sont dans le papier.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent le long de la rue mouillée. Le croissant fume encore, tout doux. À la maison, papa ouvre le sac. Le croissant est doré, un peu cassant. Tu veux un bout ? Oui, maman. S'il te plaît. Amir croque. C'est tiède. Ça sent le beurre. Merci, maman. Merci, Amir. Des miettes dorées restent au fond du sac. Tes lacets sèchent, maintenant. Ils ne tapent plus. Non. C'était celui du bout. Oui. Le paillasson, loin, garde encore la pluie. Le journal sèche, lui aussi. Il était mouillé. Un peu, oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir tire le sachet trop vite. Je le mange, d'un coup ! Le papier glisse entre les doigts. Des graines de sésame tombent au marbre. Le croissant penche vers le sol. Oh. Amir avance les mains. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Amir refuse de foncer. Personne ne dit la suite. Amir observe l'osier, écoute la boutique. Sur l'osier, un &lt;emphasis level="moderate"&gt;éclat de corbeille&lt;/emphasis&gt; brille. Là, près de la corbeille. Amir tient le sachet des deux mains. Le papier est rêche, un peu chaud. Il est chaud, papa. Tu le portes jusqu'à la porte ? Oui, papa. On sort ? Oui, maman. La porte s'ouvre. La cloche fait ding. L'air plus frais revient sur les joues. Amir serre le sachet contre lui. Il reste chaud. On marche. Le sachet penche, puis se cale. Je le tiens. On avance. Amir passe le pas de bois. Le bois craque, un peu. Les graines sont à moi. Elles sont dans le papier.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Félix croque le croissant. Maman dit &lt;emphasis&gt;merci&lt;/emphasis&gt; aussi.&lt;/slow&gt; [pause]</t>
+          <t>Amir tire le sachet trop vite. Je le mange, d'un coup ! Le papier glisse entre les doigts. Des graines de sésame tombent au marbre. Le croissant penche vers le sol. Oh. Amir avance les mains. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Amir refuse de foncer. Personne ne dit la suite. Amir observe l'osier, écoute la boutique. Sur l'osier, un &lt;emphasis&gt;éclat de corbeille&lt;/emphasis&gt; brille. Là, près de la corbeille. Amir tient le sachet des deux mains. Le papier est rêche, un peu chaud. Il est chaud, papa. Tu le portes jusqu'à la porte ? Oui, papa. On sort ? Oui, maman. La porte s'ouvre. La cloche fait ding. L'air plus frais revient sur les joues. Amir serre le sachet contre lui. Il reste chaud. On marche. Le sachet penche, puis se cale. Je le tiens. On avance. Amir passe le pas de bois. Le bois craque, un peu. Les graines sont à moi. Elles sont dans le papier. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1832,18 +1872,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1866,30 +1906,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>merci</t>
+          <t>éclat de corbeille</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1898,10 +1938,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1910,38 +1950,55 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_sans_regarder_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Ils rentrent le long de la rue mouillée.
-narrateur|Le croissant fume encore, tout doux.
-narrateur|À la maison, papa ouvre le sac.
-narrateur|Le croissant est doré, un peu cassant.
-maman|Tu veux un bout ?
+          <t>narrateur|Amir tire le sachet trop vite.
+enfant-m|Je le mange, d'un coup !
+narrateur|Le papier glisse entre les doigts.
+narrateur|Des graines de sésame tombent au marbre.
+narrateur|Le croissant penche vers le sol.
+enfant-m|Oh.
+narrateur|Amir avance les mains.
+narrateur|Puis il s'arrête net.
+enfant-m|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Amir refuse de foncer.
+narrateur|Personne ne dit la suite.
+narrateur|Amir observe l'osier, écoute la boutique.
+narrateur|Sur l'osier, un éclat de corbeille brille.
+enfant-m|Là, près de la corbeille.
+narrateur|Amir tient le sachet des deux mains.
+narrateur|Le papier est rêche, un peu chaud.
+enfant-m|Il est chaud, papa.
+papa|Tu le portes jusqu'à la porte ?
+enfant-m|Oui, papa.
+maman|On sort ?
 enfant-m|Oui, maman.
-enfant-m|S'il te plaît.
-narrateur|Amir croque.
-enfant-m|C'est tiède.
-enfant-m|Ça sent le beurre.
-enfant-m|Merci, maman.
-papa|Merci, Amir.
-narrateur|Des miettes dorées restent au fond du sac.
-maman|Tes lacets sèchent, maintenant.
-enfant-m|Ils ne tapent plus.
-papa|Non.
-maman|C'était celui du bout.
-enfant-m|Oui.
-narrateur|Le paillasson, loin, garde encore la pluie.
-papa|Le journal sèche, lui aussi.
-enfant-m|Il était mouillé.
-maman|Un peu, oui.</t>
+narrateur|La porte s'ouvre.
+narrateur|La cloche fait ding.
+narrateur|L'air plus frais revient sur les joues.
+narrateur|Amir serre le sachet contre lui.
+enfant-m|Il reste chaud.
+papa|On marche.
+narrateur|Le sachet penche, puis se cale.
+enfant-m|Je le tiens.
+maman|On avance.
+narrateur|Amir passe le pas de bois.
+narrateur|Le bois craque, un peu.
+enfant-m|Les graines sont à moi.
+maman|Elles sont dans le papier.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>pas,papier</t>
         </is>
       </c>
     </row>
@@ -1968,17 +2025,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le sac repose sur la table. Il reste une miette, encore tiède. Bonne matinée, Amir. C'était celui du bout.</t>
+          <t>L'osier brillait, papa. Tu le vois, comme dans la boutique ? Oui, sur l'osier. Amir pose le sachet contre le manteau. On le garde au chaud ? Oui, maman. Le four sentait bon. Il est contre toi. Une vapeur monte du papier. Amir respire, plus large. On rentre ? Oui. Les joues d'Amir se réchauffent. Le sachet reste tiède sous la main. Il sent le sésame. Tu le sens, près du nez ? Oui, papa. On est bien, ici. Un éclat de corbeille reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le sac repose sur la table. Il reste une miette, encore tiède. Bonne matinée, Amir. C'était celui du bout.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'osier brillait, papa. Tu le vois, comme dans la boutique ? Oui, sur l'osier. Amir pose le sachet contre le manteau. On le garde au chaud ? Oui, maman. Le four sentait bon. Il est contre toi. Une vapeur monte du papier. Amir respire, plus large. On rentre ? Oui. Les joues d'Amir se réchauffent. Le sachet reste tiède sous la main. Il sent le sésame. Tu le sens, près du nez ? Oui, papa. On est bien, ici. Un &lt;emphasis level="moderate"&gt;éclat de corbeille&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'osier brillait, papa. Tu le vois, comme dans la boutique ? Oui, sur l'osier. Amir pose le sachet contre le manteau. On le garde au chaud ? Oui, maman. Le four sentait bon. Il est contre toi. Une vapeur monte du papier. Amir respire, plus large. On rentre ? Oui. Les joues d'Amir se réchauffent. Le sachet reste tiède sous la main. Il sent le sésame. Tu le sens, près du nez ? Oui, papa. On est bien, ici. Un &lt;emphasis&gt;éclat de corbeille&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2025,7 +2082,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2033,10 +2090,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2045,12 +2102,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2059,17 +2116,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de corbeille</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2078,11 +2139,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2091,27 +2152,51 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le sac repose sur la table.
-narrateur|Il reste une miette, encore tiède.
-maman|Bonne matinée, Amir.
-papa|C'était celui du bout.</t>
+          <t>enfant-m|L'osier brillait, papa.
+papa|Tu le vois, comme dans la boutique ?
+enfant-m|Oui, sur l'osier.
+narrateur|Amir pose le sachet contre le manteau.
+maman|On le garde au chaud ?
+enfant-m|Oui, maman.
+enfant-m|Le four sentait bon.
+maman|Il est contre toi.
+narrateur|Une vapeur monte du papier.
+narrateur|Amir respire, plus large.
+papa|On rentre ?
+enfant-m|Oui.
+narrateur|Les joues d'Amir se réchauffent.
+narrateur|Le sachet reste tiède sous la main.
+enfant-m|Il sent le sésame.
+papa|Tu le sens, près du nez ?
+enfant-m|Oui, papa.
+maman|On est bien, ici.
+narrateur|Un éclat de corbeille reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pas</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2224,6 +2309,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>